<commit_message>
added vorbis excel mappings
</commit_message>
<xml_diff>
--- a/excel_files/Vorbis_ffmpeg_mapping.xlsx
+++ b/excel_files/Vorbis_ffmpeg_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MusicProcessing\excel_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDB0A60B-8898-4FD4-AD0F-E2D1F72010ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5580544C-617F-4160-948C-1FCCDF369535}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-15" yWindow="16170" windowWidth="29040" windowHeight="15840" xr2:uid="{88C1B724-2A67-4F98-976D-9A8D62A8F4F0}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="85">
   <si>
     <t>Data Type</t>
   </si>
@@ -346,15 +346,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -672,95 +670,94 @@
   <dimension ref="A1:G31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="51.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="88.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="51.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="88.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D2" s="5"/>
-      <c r="E2" s="6" t="s">
+      <c r="D2" s="4"/>
+      <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="6"/>
+      <c r="G2" s="4"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>72</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6" t="s">
+      <c r="D3" s="4"/>
+      <c r="E3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="6"/>
-      <c r="B4" s="6" t="s">
+      <c r="A4" s="4"/>
+      <c r="B4" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6" t="s">
+      <c r="D4" s="4"/>
+      <c r="E4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="4" t="s">
         <v>57</v>
       </c>
     </row>
@@ -768,323 +765,323 @@
       <c r="A5" t="s">
         <v>73</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6" t="s">
+      <c r="D5" s="4"/>
+      <c r="E5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="4" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="6"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6" t="s">
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="6"/>
+      <c r="G6" s="4"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>82</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6" t="s">
+      <c r="D7" s="4"/>
+      <c r="E7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="6"/>
+      <c r="G7" s="4"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="6"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6" t="s">
+      <c r="A8" s="4"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="6"/>
+      <c r="G8" s="4"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6" t="s">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="G9" s="6"/>
+      <c r="G9" s="4"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6" t="s">
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="6"/>
+      <c r="G10" s="4"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6" t="s">
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="G11" s="6"/>
+      <c r="G11" s="4"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="6"/>
-      <c r="B12" s="6" t="s">
+      <c r="A12" s="4"/>
+      <c r="B12" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6" t="s">
+      <c r="D12" s="4"/>
+      <c r="E12" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="G12" s="6"/>
+      <c r="G12" s="4"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>75</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6" t="s">
+      <c r="D13" s="4"/>
+      <c r="E13" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="G13" s="6"/>
+      <c r="G13" s="4"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>84</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6" t="s">
+      <c r="D14" s="4"/>
+      <c r="E14" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="G14" s="6" t="s">
+      <c r="G14" s="4" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6" t="s">
+      <c r="D15" s="4"/>
+      <c r="E15" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="G15" s="6"/>
+      <c r="G15" s="4"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>83</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6" t="s">
+      <c r="D16" s="4"/>
+      <c r="E16" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G16" s="6"/>
+      <c r="G16" s="4"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="6"/>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="7" t="s">
+      <c r="A17" s="4"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="G17" s="6"/>
+      <c r="G17" s="4"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="6"/>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6" t="s">
+      <c r="A18" s="4"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="F18" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="G18" s="6"/>
+      <c r="G18" s="4"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="6"/>
-      <c r="B19" s="6" t="s">
+      <c r="A19" s="4"/>
+      <c r="B19" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6" t="s">
+      <c r="D19" s="4"/>
+      <c r="E19" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="F19" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="G19" s="6"/>
+      <c r="G19" s="4"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="6"/>
-      <c r="B20" s="6"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6" t="s">
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="F20" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="G20" s="6"/>
+      <c r="G20" s="4"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="6"/>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="7" t="s">
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="G21" s="6"/>
+      <c r="G21" s="4"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="6"/>
-      <c r="B22" s="6"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="7" t="s">
+      <c r="A22" s="4"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="G22" s="6"/>
+      <c r="G22" s="4"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="6"/>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="7" t="s">
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="G23" s="6"/>
+      <c r="G23" s="4"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="6"/>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="7" t="s">
+      <c r="A24" s="4"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="G24" s="6"/>
+      <c r="G24" s="4"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="6"/>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="7" t="s">
+      <c r="A25" s="4"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="G25" s="6"/>
+      <c r="G25" s="4"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="6"/>
-      <c r="B26" s="6" t="s">
+      <c r="A26" s="4"/>
+      <c r="B26" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="7" t="s">
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="G26" s="6" t="s">
+      <c r="G26" s="4" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1092,72 +1089,74 @@
       <c r="A27" t="s">
         <v>74</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D27" s="6"/>
-      <c r="E27" s="6" t="s">
+      <c r="D27" s="4"/>
+      <c r="E27" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="F27" s="7" t="s">
+      <c r="F27" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="G27" s="6"/>
+      <c r="G27" s="4"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="6"/>
-      <c r="B28" s="6"/>
-      <c r="C28" s="6"/>
-      <c r="D28" s="6"/>
-      <c r="E28" s="6" t="s">
+      <c r="A28" s="4"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="F28" s="7" t="s">
+      <c r="F28" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="G28" s="6"/>
+      <c r="G28" s="4"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="6"/>
-      <c r="B29" s="6"/>
-      <c r="C29" s="6"/>
-      <c r="D29" s="6"/>
-      <c r="E29" s="6"/>
-      <c r="F29" s="7" t="s">
+      <c r="A29" s="4"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="G29" s="6"/>
+      <c r="G29" s="4"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>81</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="C30" s="6"/>
-      <c r="D30" s="6"/>
-      <c r="E30" s="6" t="s">
+      <c r="C30" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F30" s="7" t="s">
+      <c r="F30" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="G30" s="6"/>
+      <c r="G30" s="4"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="6"/>
-      <c r="B31" s="6"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
-      <c r="F31" s="7" t="s">
+      <c r="A31" s="4"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="G31" s="6"/>
+      <c r="G31" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>